<commit_message>
Fix partslink on OEM
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ELFANI\scrapper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{129A079A-D633-4D39-8604-590A7D4B0EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65593E30-C6B6-4778-8C76-A8D377D474FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{905C72F9-ABE9-4CF3-B82B-382C40698364}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Partslink</t>
   </si>
@@ -47,611 +47,29 @@
     <t>Interchange</t>
   </si>
   <si>
-    <t>101-60187</t>
+    <t>110-10005R</t>
   </si>
   <si>
-    <t>101-10026</t>
+    <t>110-10314R</t>
   </si>
   <si>
-    <t>101-10027</t>
+    <t>110-10345R</t>
   </si>
   <si>
-    <t>101-10028</t>
+    <t>MB1241164</t>
   </si>
   <si>
-    <t>101-10065</t>
+    <t>MB1241168</t>
   </si>
   <si>
-    <t>101-10066</t>
-  </si>
-  <si>
-    <t>101-10068</t>
-  </si>
-  <si>
-    <t>101-10127</t>
-  </si>
-  <si>
-    <t>101-10131</t>
-  </si>
-  <si>
-    <t>101-10146</t>
-  </si>
-  <si>
-    <t>101-10147</t>
-  </si>
-  <si>
-    <t>101-10174</t>
-  </si>
-  <si>
-    <t>101-10175</t>
-  </si>
-  <si>
-    <t>101-10176</t>
-  </si>
-  <si>
-    <t>101-10177</t>
-  </si>
-  <si>
-    <t>101-10178</t>
-  </si>
-  <si>
-    <t>101-10180</t>
-  </si>
-  <si>
-    <t>101-10181</t>
-  </si>
-  <si>
-    <t>101-10182</t>
-  </si>
-  <si>
-    <t>101-10183</t>
-  </si>
-  <si>
-    <t>101-10236</t>
-  </si>
-  <si>
-    <t>101-10239</t>
-  </si>
-  <si>
-    <t>101-10301</t>
-  </si>
-  <si>
-    <t>101-10302</t>
-  </si>
-  <si>
-    <t>101-10304</t>
-  </si>
-  <si>
-    <t>101-10397</t>
-  </si>
-  <si>
-    <t>101-10400</t>
-  </si>
-  <si>
-    <t>101-10401</t>
-  </si>
-  <si>
-    <t>101-10462</t>
-  </si>
-  <si>
-    <t>101-10591</t>
-  </si>
-  <si>
-    <t>101-10592</t>
-  </si>
-  <si>
-    <t>101-10593</t>
-  </si>
-  <si>
-    <t>101-10594</t>
-  </si>
-  <si>
-    <t>101-10595</t>
-  </si>
-  <si>
-    <t>101-10596</t>
-  </si>
-  <si>
-    <t>101-10597</t>
-  </si>
-  <si>
-    <t>101-10701</t>
-  </si>
-  <si>
-    <t>101-10702</t>
-  </si>
-  <si>
-    <t>101-10703</t>
-  </si>
-  <si>
-    <t>101-10704</t>
-  </si>
-  <si>
-    <t>101-10750</t>
-  </si>
-  <si>
-    <t>101-10752</t>
-  </si>
-  <si>
-    <t>101-10778</t>
-  </si>
-  <si>
-    <t>101-10779</t>
-  </si>
-  <si>
-    <t>101-10780</t>
-  </si>
-  <si>
-    <t>101-10787</t>
-  </si>
-  <si>
-    <t>101-10788</t>
-  </si>
-  <si>
-    <t>101-10789</t>
-  </si>
-  <si>
-    <t>101-10790</t>
-  </si>
-  <si>
-    <t>101-10791</t>
-  </si>
-  <si>
-    <t>101-10792</t>
-  </si>
-  <si>
-    <t>101-11010</t>
-  </si>
-  <si>
-    <t>101-11011</t>
-  </si>
-  <si>
-    <t>101-11102</t>
-  </si>
-  <si>
-    <t>101-11103</t>
-  </si>
-  <si>
-    <t>101-11107</t>
-  </si>
-  <si>
-    <t>101-11111</t>
-  </si>
-  <si>
-    <t>101-11124</t>
-  </si>
-  <si>
-    <t>101-11171</t>
-  </si>
-  <si>
-    <t>101-11172</t>
-  </si>
-  <si>
-    <t>101-11173</t>
-  </si>
-  <si>
-    <t>101-11175</t>
-  </si>
-  <si>
-    <t>101-11178</t>
-  </si>
-  <si>
-    <t>101-11180</t>
-  </si>
-  <si>
-    <t>101-11181</t>
-  </si>
-  <si>
-    <t>101-11438</t>
-  </si>
-  <si>
-    <t>101-11439</t>
-  </si>
-  <si>
-    <t>101-11440</t>
-  </si>
-  <si>
-    <t>101-11441</t>
-  </si>
-  <si>
-    <t>101-11497</t>
-  </si>
-  <si>
-    <t>101-11537</t>
-  </si>
-  <si>
-    <t>101-11538</t>
-  </si>
-  <si>
-    <t>101-11622</t>
-  </si>
-  <si>
-    <t>101-11624</t>
-  </si>
-  <si>
-    <t>101-11671</t>
-  </si>
-  <si>
-    <t>101-11687A</t>
-  </si>
-  <si>
-    <t>101-11687C</t>
-  </si>
-  <si>
-    <t>101-11687E</t>
-  </si>
-  <si>
-    <t>101-11706</t>
-  </si>
-  <si>
-    <t>101-11707</t>
-  </si>
-  <si>
-    <t>101-11792</t>
-  </si>
-  <si>
-    <t>101-11793</t>
-  </si>
-  <si>
-    <t>101-11794</t>
-  </si>
-  <si>
-    <t>101-11869</t>
-  </si>
-  <si>
-    <t>101-11870</t>
-  </si>
-  <si>
-    <t>101-11871</t>
-  </si>
-  <si>
-    <t>101-11872</t>
-  </si>
-  <si>
-    <t>101-11875</t>
-  </si>
-  <si>
-    <t>101-11877</t>
-  </si>
-  <si>
-    <t>101-11921</t>
-  </si>
-  <si>
-    <t>101-11922</t>
-  </si>
-  <si>
-    <t>101-11923</t>
-  </si>
-  <si>
-    <t>101-11993</t>
-  </si>
-  <si>
-    <t>101-11994</t>
-  </si>
-  <si>
-    <t>101-12014</t>
-  </si>
-  <si>
-    <t>101-12022</t>
-  </si>
-  <si>
-    <t>101-12035</t>
-  </si>
-  <si>
-    <t>101-12043</t>
-  </si>
-  <si>
-    <t>101-12044</t>
-  </si>
-  <si>
-    <t>101-12045</t>
-  </si>
-  <si>
-    <t>101-12059</t>
-  </si>
-  <si>
-    <t>101-12081</t>
-  </si>
-  <si>
-    <t>101-12111</t>
-  </si>
-  <si>
-    <t>101-12120</t>
-  </si>
-  <si>
-    <t>101-12121</t>
-  </si>
-  <si>
-    <t>101-12151</t>
-  </si>
-  <si>
-    <t>101-12152</t>
-  </si>
-  <si>
-    <t>101-12449</t>
-  </si>
-  <si>
-    <t>101-12473</t>
-  </si>
-  <si>
-    <t>101-50918C</t>
-  </si>
-  <si>
-    <t>101-50918D</t>
-  </si>
-  <si>
-    <t>101-50918H</t>
-  </si>
-  <si>
-    <t>101-50965A</t>
-  </si>
-  <si>
-    <t>101-50965C</t>
-  </si>
-  <si>
-    <t>101-51026A</t>
-  </si>
-  <si>
-    <t>101-51026D</t>
-  </si>
-  <si>
-    <t>101-51083A</t>
-  </si>
-  <si>
-    <t>101-51083C</t>
-  </si>
-  <si>
-    <t>101-51083E</t>
-  </si>
-  <si>
-    <t>101-51083G</t>
-  </si>
-  <si>
-    <t>101-51087B</t>
-  </si>
-  <si>
-    <t>101-51087D</t>
-  </si>
-  <si>
-    <t>101-51098D</t>
-  </si>
-  <si>
-    <t>101-59127E</t>
-  </si>
-  <si>
-    <t>101-59127F</t>
-  </si>
-  <si>
-    <t>101-59127G</t>
-  </si>
-  <si>
-    <t>101-59127H</t>
-  </si>
-  <si>
-    <t>101-59130A</t>
-  </si>
-  <si>
-    <t>101-59130C</t>
-  </si>
-  <si>
-    <t>101-59130D</t>
-  </si>
-  <si>
-    <t>101-59132B</t>
-  </si>
-  <si>
-    <t>101-59133A</t>
-  </si>
-  <si>
-    <t>101-59133D</t>
-  </si>
-  <si>
-    <t>101-59133E</t>
-  </si>
-  <si>
-    <t>101-59167A</t>
-  </si>
-  <si>
-    <t>101-59167C</t>
-  </si>
-  <si>
-    <t>101-59167E</t>
-  </si>
-  <si>
-    <t>101-59167F</t>
-  </si>
-  <si>
-    <t>101-59167H</t>
-  </si>
-  <si>
-    <t>101-59196B</t>
-  </si>
-  <si>
-    <t>101-59199B</t>
-  </si>
-  <si>
-    <t>101-59898A</t>
-  </si>
-  <si>
-    <t>101-59898B</t>
-  </si>
-  <si>
-    <t>101-59899A</t>
-  </si>
-  <si>
-    <t>101-59899B</t>
-  </si>
-  <si>
-    <t>101-59900A</t>
-  </si>
-  <si>
-    <t>101-59900B</t>
-  </si>
-  <si>
-    <t>101-59901A</t>
-  </si>
-  <si>
-    <t>101-59901B</t>
-  </si>
-  <si>
-    <t>101-59902A</t>
-  </si>
-  <si>
-    <t>101-59909B</t>
-  </si>
-  <si>
-    <t>101-59909C</t>
-  </si>
-  <si>
-    <t>101-59909D</t>
-  </si>
-  <si>
-    <t>101-59910B</t>
-  </si>
-  <si>
-    <t>101-59981</t>
-  </si>
-  <si>
-    <t>101-59982</t>
-  </si>
-  <si>
-    <t>101-59983</t>
-  </si>
-  <si>
-    <t>101-59984</t>
-  </si>
-  <si>
-    <t>101-59985</t>
-  </si>
-  <si>
-    <t>101-59986</t>
-  </si>
-  <si>
-    <t>101-59987</t>
-  </si>
-  <si>
-    <t>101-59988</t>
-  </si>
-  <si>
-    <t>101-60004</t>
-  </si>
-  <si>
-    <t>101-60007</t>
-  </si>
-  <si>
-    <t>101-60012</t>
-  </si>
-  <si>
-    <t>101-60013</t>
-  </si>
-  <si>
-    <t>101-60014</t>
-  </si>
-  <si>
-    <t>101-60016</t>
-  </si>
-  <si>
-    <t>101-60018</t>
-  </si>
-  <si>
-    <t>101-60026</t>
-  </si>
-  <si>
-    <t>101-60027</t>
-  </si>
-  <si>
-    <t>101-60115B</t>
-  </si>
-  <si>
-    <t>101-60170</t>
-  </si>
-  <si>
-    <t>101-60171</t>
-  </si>
-  <si>
-    <t>101-60175</t>
-  </si>
-  <si>
-    <t>101-60176</t>
-  </si>
-  <si>
-    <t>101-60177</t>
-  </si>
-  <si>
-    <t>101-60178</t>
-  </si>
-  <si>
-    <t>101-60181</t>
-  </si>
-  <si>
-    <t>101-60182</t>
-  </si>
-  <si>
-    <t>101-60183</t>
-  </si>
-  <si>
-    <t>101-60184</t>
-  </si>
-  <si>
-    <t>101-60185</t>
-  </si>
-  <si>
-    <t>101-60191</t>
-  </si>
-  <si>
-    <t>101-60231</t>
-  </si>
-  <si>
-    <t>101-60272</t>
-  </si>
-  <si>
-    <t>101-60273</t>
-  </si>
-  <si>
-    <t>101-60274</t>
-  </si>
-  <si>
-    <t>101-60276</t>
-  </si>
-  <si>
-    <t>101-60329</t>
-  </si>
-  <si>
-    <t>101-60330</t>
-  </si>
-  <si>
-    <t>101-60331</t>
-  </si>
-  <si>
-    <t>101-60333</t>
-  </si>
-  <si>
-    <t>104-10038A</t>
-  </si>
-  <si>
-    <t>104-10223A</t>
-  </si>
-  <si>
-    <t>104-10223B</t>
-  </si>
-  <si>
-    <t>104-10223C</t>
-  </si>
-  <si>
-    <t>104-10224A</t>
-  </si>
-  <si>
-    <t>101-MB1D26</t>
-  </si>
-  <si>
-    <t>101-MB1R26</t>
+    <t>MB1240172</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -664,13 +82,8 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -681,12 +94,6 @@
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -702,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -713,8 +120,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1065,1224 +470,639 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-      <c r="B2" s="4" t="s">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="4" t="s">
-        <v>200</v>
+      <c r="A3" t="s">
+        <v>6</v>
       </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="4" t="s">
-        <v>201</v>
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
-      <c r="B5" s="4" t="s">
-        <v>3</v>
-      </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
-      <c r="B6" s="4" t="s">
-        <v>4</v>
-      </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
-      <c r="B7" s="4" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
-      <c r="B8" s="4" t="s">
-        <v>6</v>
-      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
-      <c r="B9" s="4" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
-      <c r="B10" s="4" t="s">
-        <v>8</v>
-      </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="4" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
-      <c r="B12" s="4" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
-      <c r="B13" s="4" t="s">
-        <v>11</v>
-      </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
-      <c r="B14" s="4" t="s">
-        <v>12</v>
-      </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
-      <c r="B15" s="4" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
-      <c r="B16" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
-      <c r="B17" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
-      <c r="B18" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
-      <c r="B19" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
-      <c r="B24" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
-      <c r="B26" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
-      <c r="B28" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
-      <c r="B29" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
-      <c r="B30" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
-      <c r="B31" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
-      <c r="B32" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
-      <c r="B33" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
-      <c r="B34" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
-      <c r="B35" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
-      <c r="B36" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
-      <c r="B37" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
-      <c r="B38" s="4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
-      <c r="B39" s="4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
-      <c r="B40" s="4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="2"/>
-      <c r="B41" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
-      <c r="B42" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
-      <c r="B43" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="2"/>
-      <c r="B44" s="4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="2"/>
-      <c r="B45" s="4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="2"/>
-      <c r="B46" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="2"/>
-      <c r="B47" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="2"/>
-      <c r="B48" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="2"/>
-      <c r="B49" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" s="2"/>
-      <c r="B50" s="4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="2"/>
-      <c r="B51" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="2"/>
-      <c r="B52" s="4" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="2"/>
-      <c r="B53" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="2"/>
-      <c r="B54" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" s="2"/>
-      <c r="B55" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" s="2"/>
-      <c r="B56" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="2"/>
-      <c r="B57" s="4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="2"/>
-      <c r="B58" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" s="2"/>
-      <c r="B59" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" s="2"/>
-      <c r="B60" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" s="2"/>
-      <c r="B61" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" s="2"/>
-      <c r="B62" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" s="2"/>
-      <c r="B63" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" s="2"/>
-      <c r="B64" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" s="2"/>
-      <c r="B65" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" s="2"/>
-      <c r="B66" s="4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="2"/>
-      <c r="B67" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="2"/>
-      <c r="B68" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" s="2"/>
-      <c r="B69" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" s="2"/>
-      <c r="B70" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" s="2"/>
-      <c r="B71" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" s="2"/>
-      <c r="B72" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" s="2"/>
-      <c r="B73" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" s="2"/>
-      <c r="B74" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" s="2"/>
-      <c r="B75" s="4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" s="2"/>
-      <c r="B76" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" s="2"/>
-      <c r="B77" s="4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" s="2"/>
-      <c r="B78" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" s="2"/>
-      <c r="B79" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" s="2"/>
-      <c r="B80" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" s="2"/>
-      <c r="B81" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" s="2"/>
-      <c r="B82" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="2"/>
-      <c r="B83" s="4" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" s="2"/>
-      <c r="B84" s="4" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" s="2"/>
-      <c r="B85" s="4" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" s="2"/>
-      <c r="B86" s="4" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" s="2"/>
-      <c r="B87" s="4" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" s="2"/>
-      <c r="B88" s="4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" s="2"/>
-      <c r="B89" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" s="2"/>
-      <c r="B90" s="4" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" s="2"/>
-      <c r="B91" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A92" s="2"/>
-      <c r="B92" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" s="2"/>
-      <c r="B93" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" s="2"/>
-      <c r="B94" s="4" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" s="2"/>
-      <c r="B95" s="4" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" s="2"/>
-      <c r="B96" s="4" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" s="2"/>
-      <c r="B97" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" s="2"/>
-      <c r="B98" s="4" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" s="2"/>
-      <c r="B99" s="4" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" s="2"/>
-      <c r="B100" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" s="2"/>
-      <c r="B101" s="4" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" s="2"/>
-      <c r="B102" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" s="2"/>
-      <c r="B103" s="4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" s="2"/>
-      <c r="B104" s="4" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" s="2"/>
-      <c r="B105" s="4" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" s="2"/>
-      <c r="B106" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" s="2"/>
-      <c r="B107" s="4" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" s="2"/>
-      <c r="B108" s="4" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" s="2"/>
-      <c r="B109" s="4" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A110" s="2"/>
-      <c r="B110" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" s="2"/>
-      <c r="B111" s="4" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" s="2"/>
-      <c r="B112" s="4" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" s="2"/>
-      <c r="B113" s="5" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" s="2"/>
-      <c r="B114" s="5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" s="2"/>
-      <c r="B115" s="5" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A116" s="2"/>
-      <c r="B116" s="5" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A117" s="2"/>
-      <c r="B117" s="5" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A118" s="2"/>
-      <c r="B118" s="5" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A119" s="2"/>
-      <c r="B119" s="5" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A120" s="2"/>
-      <c r="B120" s="4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A121" s="2"/>
-      <c r="B121" s="4" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A122" s="2"/>
-      <c r="B122" s="4" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A123" s="2"/>
-      <c r="B123" s="4" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A124" s="2"/>
-      <c r="B124" s="4" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A125" s="2"/>
-      <c r="B125" s="4" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A126" s="2"/>
-      <c r="B126" s="4" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A127" s="2"/>
-      <c r="B127" s="4" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A128" s="2"/>
-      <c r="B128" s="4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A129" s="2"/>
-      <c r="B129" s="4" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A130" s="2"/>
-      <c r="B130" s="4" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A131" s="2"/>
-      <c r="B131" s="4" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A132" s="2"/>
-      <c r="B132" s="4" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A133" s="2"/>
-      <c r="B133" s="5" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A134" s="2"/>
-      <c r="B134" s="4" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A135" s="2"/>
-      <c r="B135" s="4" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A136" s="2"/>
-      <c r="B136" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A137" s="2"/>
-      <c r="B137" s="4" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A138" s="2"/>
-      <c r="B138" s="4" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A139" s="2"/>
-      <c r="B139" s="5" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A140" s="2"/>
-      <c r="B140" s="4" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A141" s="2"/>
-      <c r="B141" s="4" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A142" s="2"/>
-      <c r="B142" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A143" s="2"/>
-      <c r="B143" s="4" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A144" s="2"/>
-      <c r="B144" s="4" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A145" s="2"/>
-      <c r="B145" s="4" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="146" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A146" s="2"/>
-      <c r="B146" s="4" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="147" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A147" s="2"/>
-      <c r="B147" s="4" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="148" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A148" s="2"/>
-      <c r="B148" s="5" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="149" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A149" s="2"/>
-      <c r="B149" s="4" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="150" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A150" s="2"/>
-      <c r="B150" s="4" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="151" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A151" s="2"/>
-      <c r="B151" s="4" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A152" s="2"/>
-      <c r="B152" s="4" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A153" s="2"/>
-      <c r="B153" s="4" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A154" s="2"/>
-      <c r="B154" s="4" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A155" s="2"/>
-      <c r="B155" s="5" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A156" s="2"/>
-      <c r="B156" s="4" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A157" s="2"/>
-      <c r="B157" s="4" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A158" s="2"/>
-      <c r="B158" s="4" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A159" s="2"/>
-      <c r="B159" s="5" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="160" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A160" s="2"/>
-      <c r="B160" s="4" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A161" s="2"/>
-      <c r="B161" s="4" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="162" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A162" s="2"/>
-      <c r="B162" s="4" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="163" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A163" s="2"/>
-      <c r="B163" s="5" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="164" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A164" s="2"/>
-      <c r="B164" s="5" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="165" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A165" s="2"/>
-      <c r="B165" s="4" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="166" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A166" s="2"/>
-      <c r="B166" s="4" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="167" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A167" s="2"/>
-      <c r="B167" s="4" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="168" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A168" s="2"/>
-      <c r="B168" s="4" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="169" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A169" s="2"/>
-      <c r="B169" s="5" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="170" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A170" s="2"/>
-      <c r="B170" s="5" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="171" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A171" s="2"/>
-      <c r="B171" s="4" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="172" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A172" s="2"/>
-      <c r="B172" s="4" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="173" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A173" s="2"/>
-      <c r="B173" s="4" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="174" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A174" s="2"/>
-      <c r="B174" s="4" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="175" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A175" s="2"/>
-      <c r="B175" s="4" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="176" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A176" s="2"/>
-      <c r="B176" s="4" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="177" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A177" s="2"/>
-      <c r="B177" s="4" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="178" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A178" s="2"/>
-      <c r="B178" s="4" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="179" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A179" s="2"/>
-      <c r="B179" s="4" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="180" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A180" s="2"/>
-      <c r="B180" s="4" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="181" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A181" s="2"/>
-      <c r="B181" s="4" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="182" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A182" s="2"/>
-      <c r="B182" s="4" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A183" s="2"/>
-      <c r="B183" s="5" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A184" s="2"/>
-      <c r="B184" s="4" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="185" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A185" s="2"/>
-      <c r="B185" s="4" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="186" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A186" s="2"/>
-      <c r="B186" s="5" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="187" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A187" s="2"/>
-      <c r="B187" s="4" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="188" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A188" s="2"/>
-      <c r="B188" s="5" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="189" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A189" s="2"/>
-      <c r="B189" s="4" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="190" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A190" s="2"/>
-      <c r="B190" s="4" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="191" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="191" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A191" s="2"/>
-      <c r="B191" s="4" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="192" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A192" s="2"/>
-      <c r="B192" s="4" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="193" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A193" s="2"/>
-      <c r="B193" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="194" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A194" s="2"/>
-      <c r="B194" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="195" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A195" s="2"/>
-      <c r="B195" s="4" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="196" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A196" s="2"/>
-      <c r="B196" s="4" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="197" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A197" s="2"/>
-      <c r="B197" s="4" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="198" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A198" s="2"/>
-      <c r="B198" s="4" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="199" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A199" s="2"/>
-      <c r="B199" s="4" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="200" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A200" s="2"/>
-      <c r="B200" s="4" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="201" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A201" s="2"/>
-      <c r="B201" s="4" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="202" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A202" s="2"/>
     </row>
-    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A203" s="2"/>
     </row>
-    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A204" s="2"/>
     </row>
-    <row r="205" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A205" s="2"/>
     </row>
-    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A206" s="2"/>
     </row>
-    <row r="207" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A207" s="2"/>
     </row>
-    <row r="208" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A208" s="2"/>
     </row>
     <row r="209" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>